<commit_message>
primera version del modulo para manejar excel
</commit_message>
<xml_diff>
--- a/app/fixtures/excel_ejemplo.xlsx
+++ b/app/fixtures/excel_ejemplo.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ventas!$A$3:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Movimientos!$A$3:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Movimientos!$A$3:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Ventas!$A$3:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Movimientos!$A$3:$F$15</definedName>
   </definedNames>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t xml:space="preserve">Registro Detallado de Ventas</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Promociones</t>
   </si>
   <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
     <t xml:space="preserve">Registro de Movimientos Financieros</t>
   </si>
   <si>
@@ -198,12 +195,6 @@
   </si>
   <si>
     <t xml:space="preserve">Reparación de equipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Ingresos:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total Gastos:</t>
   </si>
 </sst>
 </file>
@@ -255,7 +246,7 @@
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -272,6 +263,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="0"/>
+        <bgColor theme="0" tint="0"/>
       </patternFill>
     </fill>
     <fill>
@@ -358,12 +355,12 @@
     <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="2" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
+    <xf fontId="4" fillId="4" borderId="2" numFmtId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
     <xf fontId="4" fillId="0" borderId="2" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" quotePrefix="0" pivotButton="0"/>
-    <xf fontId="5" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="5" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="6" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
+    <xf fontId="6" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="0" pivotButton="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1135,17 +1132,9 @@
       </c>
     </row>
     <row r="14" ht="15.75">
-      <c r="C14" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="16">
-        <f>SUM(D4:D13)</f>
-        <v>95</v>
-      </c>
-      <c r="F14" s="17">
-        <f>SUM(F4:F13)</f>
-        <v>335.5</v>
-      </c>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="F14" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F13"/>
@@ -1162,7 +1151,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="14"/>
     <col customWidth="1" min="2" max="2" width="12"/>
@@ -1174,7 +1163,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
@@ -1182,238 +1171,228 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4">
+    </row>
+    <row r="4" ht="15">
       <c r="A4" s="10" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="E4" s="14">
         <v>125</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" ht="15">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="11" t="s">
         <v>41</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>42</v>
       </c>
       <c r="E5" s="14">
         <v>80</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" ht="15">
       <c r="A6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E6" s="14">
         <v>70</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" ht="15">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C7" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>46</v>
       </c>
       <c r="E7" s="14">
         <v>45</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" ht="15">
       <c r="A8" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C8" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="11" t="s">
         <v>47</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>48</v>
       </c>
       <c r="E8" s="14">
         <v>30</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" ht="15">
       <c r="A9" s="10" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>49</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>50</v>
       </c>
       <c r="E9" s="14">
         <v>20</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" ht="15">
       <c r="A10" s="10" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="E10" s="14">
         <v>25</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" ht="15">
       <c r="A11" s="10" t="s">
         <v>21</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>54</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>55</v>
       </c>
       <c r="E11" s="14">
         <v>250</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="12">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" ht="15">
       <c r="A12" s="10" t="s">
         <v>23</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="D12" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="E12" s="14">
         <v>180</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13" ht="15">
       <c r="A13" s="10" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="E13" s="14">
         <v>40</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="D14" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="17">
-        <f>SUMIF(B4:B13,"Ingreso",E4:E13)</f>
-        <v>405</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="D15" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="E15" s="17">
-        <f>SUMIF(B4:B13,"Gasto",E4:E13)</f>
-        <v>460</v>
-      </c>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75">
+      <c r="D14" s="15"/>
+      <c r="E14" s="17"/>
+    </row>
+    <row r="15" ht="15.75">
+      <c r="D15" s="15"/>
+      <c r="E15" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:F15"/>

</xml_diff>